<commit_message>
Sprint 3 nhóm chủ quán: mã giảm giá, tính tiền theo bàn, đánh giá
- FR-46: chủ quán tạo/sửa/tắt/xóa mã giảm giá (% hoặc số tiền, đơn tối thiểu, hạn, số lượt)
- FR-23: khách nhập mã ở giỏ hàng; server tính giảm giá (POST /api/orders/quote), giữ lượt dùng nguyên tử, trả lượt khi hủy đơn
- FR-45: trang tính tiền theo bàn, thu tiền cả bàn (POST /api/tables/<id>/settle)
- FR-24/FR-49: khách đánh giá đơn hoàn thành bằng mã đơn (một lần/đơn); chủ quán xem điểm trung bình, phân bố sao, nhận xét
- Dữ liệu mẫu có mã giảm giá, đơn giảm giá và đánh giá; 18 test mới (tổng 88)
- Cập nhật README và trạng thái FR/US

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KmcifPk7biQekxyaV5upbh
</commit_message>
<xml_diff>
--- a/docs/Danh_sach_chuc_nang_QuickOrder.xlsx
+++ b/docs/Danh_sach_chuc_nang_QuickOrder.xlsx
@@ -1806,7 +1806,7 @@
       </c>
       <c r="L20" s="25" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1868,7 +1868,7 @@
       </c>
       <c r="L21" s="25" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -3034,7 +3034,7 @@
       </c>
       <c r="L40" s="25" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -3092,7 +3092,7 @@
       </c>
       <c r="L41" s="25" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -3270,7 +3270,7 @@
       </c>
       <c r="L44" s="25" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: cập nhật tài liệu sau Sprint 3
- README: trạng thái Sprint 3, tính năng, cấu trúc thư mục, bảng endpoint, kết quả 152 test, hướng dẫn kiểm tra nhanh
- sequence_diagram.md: viết lại theo API thực tế đến hết Sprint 3
- Danh sách chức năng: 48/49 hoàn thành (còn FR-27, Mở rộng)
- User Story: 50/51 hoàn thành (còn US-24, Mở rộng)
- RouteAPI v1.1: thêm mục 9 liệt kê API JSON đã triển khai

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QUC6HUnL43YxjV2v3TcRX9
</commit_message>
<xml_diff>
--- a/docs/Danh_sach_chuc_nang_QuickOrder.xlsx
+++ b/docs/Danh_sach_chuc_nang_QuickOrder.xlsx
@@ -1667,7 +1667,7 @@
       </c>
       <c r="I18" s="23" t="inlineStr">
         <is>
-          <t>Cần đăng nhập vì khách ẩn danh không có lịch sử.</t>
+          <t>Cần đăng nhập vì khách ẩn danh không có lịch sử. Đơn đặt khi đã đăng nhập tự vào lịch sử; đơn đặt trước đó có thể lưu vào tài khoản bằng mã riêng của đơn trên đúng trình duyệt đã đặt.</t>
         </is>
       </c>
       <c r="J18" s="25" t="inlineStr">
@@ -1682,7 +1682,7 @@
       </c>
       <c r="L18" s="25" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1744,7 +1744,7 @@
       </c>
       <c r="L19" s="25" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1930,7 +1930,7 @@
       </c>
       <c r="L22" s="25" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -1977,7 +1977,7 @@
       </c>
       <c r="I23" s="23" t="inlineStr">
         <is>
-          <t>Bổ sung: để Admin có đầu vào cho FR-55.</t>
+          <t>Bổ sung: để chủ quán có đầu vào cho FR-55. Nội dung 10 đến 500 ký tự; chỉ gửi được khi đơn đã qua bước chờ xác nhận; mỗi đơn tối đa 5 khiếu nại, và chỉ có một khiếu nại chưa đóng tại một thời điểm. Khách ẩn danh gửi bằng mã riêng của đơn.</t>
         </is>
       </c>
       <c r="J23" s="25" t="inlineStr">
@@ -1992,7 +1992,7 @@
       </c>
       <c r="L23" s="25" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -3150,7 +3150,7 @@
       </c>
       <c r="L42" s="25" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -3208,7 +3208,7 @@
       </c>
       <c r="L43" s="25" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -3390,7 +3390,7 @@
       </c>
       <c r="L46" s="25" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -3448,7 +3448,7 @@
       </c>
       <c r="L47" s="25" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -3510,7 +3510,7 @@
       </c>
       <c r="L48" s="25" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -3555,7 +3555,11 @@
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="I49" s="23" t="n"/>
+      <c r="I49" s="23" t="inlineStr">
+        <is>
+          <t>Số liệu toàn bộ thời gian (chưa lọc theo khoảng thời gian). Doanh thu chỉ tính đơn Hoàn thành.</t>
+        </is>
+      </c>
       <c r="J49" s="25" t="inlineStr">
         <is>
           <t>UC-40</t>
@@ -3568,7 +3572,7 @@
       </c>
       <c r="L49" s="25" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>
@@ -3580,7 +3584,7 @@
       </c>
       <c r="B50" s="23" t="inlineStr">
         <is>
-          <t>Quản trị viên</t>
+          <t>Chủ quán</t>
         </is>
       </c>
       <c r="C50" s="23" t="inlineStr">
@@ -3595,12 +3599,12 @@
       </c>
       <c r="E50" s="23" t="inlineStr">
         <is>
-          <t>Xem khiếu nại của khách, phản hồi và đóng khiếu nại.</t>
+          <t>Chủ quán xem khiếu nại của khách về các quán của mình, phản hồi và đóng khiếu nại.</t>
         </is>
       </c>
       <c r="F50" s="23" t="inlineStr">
         <is>
-          <t>Quản trị viên</t>
+          <t>Chủ quán</t>
         </is>
       </c>
       <c r="G50" s="25" t="inlineStr">
@@ -3615,7 +3619,7 @@
       </c>
       <c r="I50" s="23" t="inlineStr">
         <is>
-          <t>Phụ thuộc FR-26.</t>
+          <t>Phụ thuộc FR-26. Chốt ở Sprint 3: chủ quán xử lý khiếu nại của quán mình; chủ quán khác và quản trị viên không có API xem hay sửa khiếu nại này. Phải lưu phản hồi trước khi đóng.</t>
         </is>
       </c>
       <c r="J50" s="25" t="inlineStr">
@@ -3630,7 +3634,7 @@
       </c>
       <c r="L50" s="25" t="inlineStr">
         <is>
-          <t>Chưa làm</t>
+          <t>Hoàn thành</t>
         </is>
       </c>
     </row>

</xml_diff>